<commit_message>
Upd(be): crane data to suit updated crane model
</commit_message>
<xml_diff>
--- a/backend/data/attachments/crawler/Liebherr_LR1100.xlsx
+++ b/backend/data/attachments/crawler/Liebherr_LR1100.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\crane_lifting_capacity\data\crawler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F924106E-0C59-48B4-83C2-89B94D336D58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E2DBE8F-C131-4658-97DF-E0B322935C22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-6060" windowWidth="29040" windowHeight="15840" xr2:uid="{D0CD5142-251E-41F7-B82A-77810B023ACC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{D0CD5142-251E-41F7-B82A-77810B023ACC}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="18" r:id="rId1"/>
@@ -43,9 +43,6 @@
   </si>
   <si>
     <t>-</t>
-  </si>
-  <si>
-    <t>crawler</t>
   </si>
   <si>
     <t>LR1100</t>
@@ -85,6 +82,9 @@
   </si>
   <si>
     <t>Максимальная грузоподъемность</t>
+  </si>
+  <si>
+    <t>Гусеничный</t>
   </si>
 </sst>
 </file>
@@ -789,21 +789,21 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D1" s="27" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D2" s="27">
         <v>4722</v>
@@ -811,21 +811,21 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="D3" s="27" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>12</v>
       </c>
       <c r="D4" s="27">
         <v>1064.54</v>
@@ -833,22 +833,21 @@
     </row>
     <row r="5" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>14</v>
-      </c>
       <c r="D5" s="27" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G5" s="28">
-        <f>C9</f>
         <v>104.5</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="29" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C6" s="30"/>
       <c r="D6" s="30"/>

</xml_diff>